<commit_message>
Upgrade analytics methodology and runnable dbt pipeline
</commit_message>
<xml_diff>
--- a/artifacts/finance_analysis.xlsx
+++ b/artifacts/finance_analysis.xlsx
@@ -10,8 +10,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Detail" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Logistics Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Detail" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Executive Summary'!$A$3:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Market Detail'!$A$1:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Logistics Detail'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Experiment Detail'!$A$1:$L$3</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -174,7 +180,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Executive Summary'!D3</f>
+              <f>'Executive Summary'!E3</f>
             </strRef>
           </tx>
           <spPr>
@@ -189,7 +195,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Executive Summary'!$D$4:$D$8</f>
+              <f>'Executive Summary'!$E$4:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -233,7 +239,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>7</col>
       <colOff>0</colOff>
       <row>2</row>
       <rowOff>0</rowOff>
@@ -545,8 +551,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -555,6 +569,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -563,99 +578,116 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Orders</t>
+          <t>Prospects</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Conversion</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Net Revenue</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Contribution Margin</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Margin %</t>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Margin/Prospect</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>836</v>
+        <v>1031</v>
       </c>
       <c r="C4" t="n">
-        <v>48115.09</v>
+        <v>0.4267</v>
       </c>
       <c r="D4" t="n">
-        <v>6628.04</v>
+        <v>28672.99</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1378</v>
+        <v>3496.25</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3.39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>702</v>
+        <v>1202</v>
       </c>
       <c r="C5" t="n">
-        <v>38536.55</v>
+        <v>0.3924</v>
       </c>
       <c r="D5" t="n">
-        <v>5178.46</v>
+        <v>28736.89</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1344</v>
+        <v>2808.39</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Affiliate</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1067</v>
+        <v>701</v>
       </c>
       <c r="C6" t="n">
-        <v>60382.9</v>
+        <v>0.3225</v>
       </c>
       <c r="D6" t="n">
-        <v>207.49</v>
+        <v>14377.64</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0034</v>
+        <v>-323.09</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Affiliate</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>463</v>
+        <v>1549</v>
       </c>
       <c r="C7" t="n">
-        <v>24725.16</v>
+        <v>0.4522</v>
       </c>
       <c r="D7" t="n">
-        <v>-326.44</v>
+        <v>43804.53</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0132</v>
+        <v>-3044.04</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-1.97</v>
       </c>
     </row>
     <row r="8">
@@ -665,22 +697,38 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>823</v>
+        <v>1517</v>
       </c>
       <c r="C8" t="n">
-        <v>44845.42</v>
+        <v>0.2949</v>
       </c>
       <c r="D8" t="n">
-        <v>-6612.55</v>
+        <v>28118.53</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.1475</v>
+        <v>-3965.57</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-2.61</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:F8"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <conditionalFormatting sqref="E4:E8">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -694,6 +742,13 @@
   </sheetPr>
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
@@ -729,16 +784,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1973</v>
+        <v>1262</v>
       </c>
       <c r="C2" t="n">
-        <v>110098.71</v>
+        <v>70108.41</v>
       </c>
       <c r="D2" t="n">
-        <v>3671.47</v>
+        <v>447.06</v>
       </c>
       <c r="E2" t="n">
-        <v>1.86</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="3">
@@ -748,16 +803,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>796</v>
+        <v>504</v>
       </c>
       <c r="C3" t="n">
-        <v>43318.17</v>
+        <v>30747.85</v>
       </c>
       <c r="D3" t="n">
-        <v>711.1799999999999</v>
+        <v>-168.5</v>
       </c>
       <c r="E3" t="n">
-        <v>0.89</v>
+        <v>-0.33</v>
       </c>
     </row>
     <row r="4">
@@ -767,19 +822,20 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1122</v>
+        <v>812</v>
       </c>
       <c r="C4" t="n">
-        <v>63188.24</v>
+        <v>42854.32</v>
       </c>
       <c r="D4" t="n">
-        <v>692.35</v>
+        <v>-1306.62</v>
       </c>
       <c r="E4" t="n">
-        <v>0.62</v>
+        <v>-1.61</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -790,8 +846,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
@@ -801,15 +864,20 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>deliveries</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>on_time_rate</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>avg_delivery_cost</t>
         </is>
@@ -818,17 +886,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FastShip</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1304</v>
+          <t>BalticPost</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>EE</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9578</v>
+        <v>212</v>
       </c>
       <c r="D2" t="n">
-        <v>5.52</v>
+        <v>0.8585</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5.41</v>
       </c>
     </row>
     <row r="3">
@@ -837,33 +910,341 @@
           <t>BalticPost</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>1738</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>0.916</v>
+        <v>367</v>
       </c>
       <c r="D3" t="n">
-        <v>4.58</v>
+        <v>0.8992</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>BalticPost</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>544</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4.14</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>EconomyBox</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>849</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.7845</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3.97</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EE</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>116</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.8621</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EconomyBox</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>168</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EconomyBox</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>291</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.8763</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3.54</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FastShip</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>EE</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>176</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="E8" t="n">
+        <v>6.42</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FastShip</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>277</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.9711</v>
+      </c>
+      <c r="E9" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FastShip</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>427</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.9649</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>treatment</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>assigned_prospects</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>converted_prospects</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>conversion_rate</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>margin_per_assigned_prospect</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>revenue_per_assigned_prospect</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>conversion_lift_pp</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>conversion_ci_low_pp</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>conversion_ci_high_pp</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>conversion_p_value</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>margin_lift_vs_control</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>srm_p_value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>control</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3006</v>
+      </c>
+      <c r="C2" t="n">
+        <v>864</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.2874</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="F2" t="n">
+        <v>22.51</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="I2" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="K2" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.8769</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>treatment</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2994</v>
+      </c>
+      <c r="C3" t="n">
+        <v>973</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-0.71</v>
+      </c>
+      <c r="F3" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="I3" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="K3" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.8769</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>